<commit_message>
refactored the cumilative import
</commit_message>
<xml_diff>
--- a/sheets/TARGET  SHEET 2024-25 NEW (1).xlsx
+++ b/sheets/TARGET  SHEET 2024-25 NEW (1).xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\OneDrive\Desktop\sheets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F55DBA2-3FBB-4E53-BEF2-609AEF4D582B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8D3A4EE-9214-459B-93A7-435840F8A1FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="XA" sheetId="1" r:id="rId1"/>
@@ -4492,7 +4492,7 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-IN"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -4565,7 +4565,7 @@
                     <a:latin typeface="+mn-lt"/>
                   </a:defRPr>
                 </a:pPr>
-                <a:endParaRPr/>
+                <a:endParaRPr lang="en-IN"/>
               </a:p>
             </c:rich>
           </c:tx>
@@ -5288,7 +5288,9 @@
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="15" customWidth="1"/>
     <col min="3" max="3" width="30.109375" customWidth="1"/>
-    <col min="4" max="26" width="8" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" customWidth="1"/>
+    <col min="5" max="5" width="24.77734375" customWidth="1"/>
+    <col min="6" max="26" width="8" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="45" customHeight="1" x14ac:dyDescent="0.3">

</xml_diff>